<commit_message>
feat: harden salary workflows and customer phone imports
</commit_message>
<xml_diff>
--- a/docs/OS_PLUS_QA_Test_Matrix.xlsx
+++ b/docs/OS_PLUS_QA_Test_Matrix.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Access" sheetId="1" r:id="Rda433e07ac304f3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles Permissions" sheetId="2" r:id="R5b3166cfb8654d5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Isolation" sheetId="3" r:id="Rf5786b573b2d4f2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="4" r:id="Ref99ef6dc20d489a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="5" r:id="Rb4f72f9753d84c82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuration" sheetId="6" r:id="R1a736571103c425a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="7" r:id="R0f9bbdd89766400b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="8" r:id="Rcff5f175c69845ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worker Contributions" sheetId="9" r:id="Rded4f65d623b4f99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="10" r:id="R58f4c2404dba4177"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform UX" sheetId="11" r:id="R483820667ae94283"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary" sheetId="12" r:id="R4e3937ce22ac43de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="13" r:id="R196ea2650d9c43f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attachments" sheetId="14" r:id="R73b74199c0884ea5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Communications" sheetId="15" r:id="Rcbbea6649fce437c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Tracking" sheetId="16" r:id="Rf501bac7686c40a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Smoke" sheetId="17" r:id="R58e3027d51464f79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Access" sheetId="1" r:id="R7a255d7c452f4804"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles Permissions" sheetId="2" r:id="Rc737d018cea5457b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Isolation" sheetId="3" r:id="Rfcc05599e8984119"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="4" r:id="Rb59d4bafdc7245b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="5" r:id="Rb7cce644c1d74a28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuration" sheetId="6" r:id="Rd4e02d6ab2f14490"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="7" r:id="Rfe2e6ec88a604fe7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="8" r:id="Rb5549c3c50544f75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worker Contributions" sheetId="9" r:id="Rb89bc9b0b1984937"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="10" r:id="Rdc8c349c453245b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform UX" sheetId="11" r:id="R1dd35a1edee64337"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary" sheetId="12" r:id="R7aeede8cbbfa45e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="13" r:id="Rb3a73360f23b44e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attachments" sheetId="14" r:id="R724d511d9a574958"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Communications" sheetId="15" r:id="R0a9df2737d5b4a00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Tracking" sheetId="16" r:id="R2e172924c85e4347"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Smoke" sheetId="17" r:id="R4305f313d4124e1c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -169,7 +169,7 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="SalaryTable" displayName="SalaryTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="SalaryTable" displayName="SalaryTable" ref="A1:K21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -188,7 +188,7 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="FinanceTable" displayName="FinanceTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="FinanceTable" displayName="FinanceTable" ref="A1:K6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -359,7 +359,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ConfigurationTable" displayName="ConfigurationTable" ref="A1:K12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ConfigurationTable" displayName="ConfigurationTable" ref="A1:K13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -812,7 +812,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad27cad41c6e415e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdef80c8aa9134677"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1248,7 +1248,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfe559891e8e49c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56e449a81e824c3d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1494,7 +1494,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a9423a216654633"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7bf2df2c10043e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1644,10 +1644,541 @@
       </x:c>
       <x:c r="K4" s="6" t="str"/>
     </x:row>
+    <x:row r="5" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>SA-004</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E5" s="6" t="str">
+        <x:v>A salary period contains at least two unpaid workers and active payment modes.</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="str">
+        <x:v>Record one worker payment from the period workspace.</x:v>
+      </x:c>
+      <x:c r="G5" s="6" t="str">
+        <x:v>Success remains in the same period with the same worker expanded; the next worker can be paid without returning through Overview.</x:v>
+      </x:c>
+      <x:c r="H5" s="6" t="str"/>
+      <x:c r="I5" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J5" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K5" s="6" t="str"/>
+    </x:row>
+    <x:row r="6" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>SA-005</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E6" s="6" t="str">
+        <x:v>A worker has no advance or loan balance.</x:v>
+      </x:c>
+      <x:c r="F6" s="6" t="str">
+        <x:v>Attempt a repayment or salary deduction, then issue an advance and repeat with an amount above and within the balance.</x:v>
+      </x:c>
+      <x:c r="G6" s="6" t="str">
+        <x:v>Missing account and over-balance commands fail atomically; the valid amount succeeds and cannot make the selected balance negative.</x:v>
+      </x:c>
+      <x:c r="H6" s="6" t="str"/>
+      <x:c r="I6" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J6" s="6" t="str">
+        <x:v>Database + Automated</x:v>
+      </x:c>
+      <x:c r="K6" s="6" t="str"/>
+    </x:row>
+    <x:row r="7" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>SA-006</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E7" s="6" t="str">
+        <x:v>Active payment modes and worker exist.</x:v>
+      </x:c>
+      <x:c r="F7" s="6" t="str">
+        <x:v>Record an advance, loan, cash repayment, salary deduction, salary credit, and salary payment; generate or regenerate a draft suggestion covering the entry date and inspect cash classifications plus an existing finalized payable.</x:v>
+      </x:c>
+      <x:c r="G7" s="6" t="str">
+        <x:v>Advance/loan/payment are cash out, repayment is cash in, deduction/credit are non-cash; only deduction and credit affect the generated/regenerated suggestion, and the existing founder-finalized payable is unchanged.</x:v>
+      </x:c>
+      <x:c r="H7" s="6" t="str"/>
+      <x:c r="I7" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J7" s="6" t="str">
+        <x:v>Database + Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K7" s="6" t="str">
+        <x:v>Advance/loan issuance is never automatically deducted from salary.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>SA-007</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E8" s="6" t="str">
+        <x:v>A valid worker-money form is ready.</x:v>
+      </x:c>
+      <x:c r="F8" s="6" t="str">
+        <x:v>Submit the same idempotency key twice or retry after a network interruption.</x:v>
+      </x:c>
+      <x:c r="G8" s="6" t="str">
+        <x:v>Exactly one active ledger entry is created and balances/cash totals are not duplicated.</x:v>
+      </x:c>
+      <x:c r="H8" s="6" t="str"/>
+      <x:c r="I8" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J8" s="6" t="str">
+        <x:v>Database + Automated</x:v>
+      </x:c>
+      <x:c r="K8" s="6" t="str"/>
+    </x:row>
+    <x:row r="9" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>SA-008</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="str">
+        <x:v>Owner/Admin</x:v>
+      </x:c>
+      <x:c r="D9" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E9" s="6" t="str">
+        <x:v>An active advance/loan/payment entry exists.</x:v>
+      </x:c>
+      <x:c r="F9" s="6" t="str">
+        <x:v>Correct the entry with a reason, then reverse another entry with a reason.</x:v>
+      </x:c>
+      <x:c r="G9" s="6" t="str">
+        <x:v>Original history remains visible; replacement links to the original; reversed rows stop affecting balances, salary, and Finance exactly once.</x:v>
+      </x:c>
+      <x:c r="H9" s="6" t="str"/>
+      <x:c r="I9" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J9" s="6" t="str">
+        <x:v>Database + Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K9" s="6" t="str">
+        <x:v>Issuance correction/reversal is blocked if it would make a balance negative.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A10" s="6" t="str">
+        <x:v>SA-009</x:v>
+      </x:c>
+      <x:c r="B10" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C10" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D10" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E10" s="6" t="str">
+        <x:v>Manager membership is active and worker-money entries exist.</x:v>
+      </x:c>
+      <x:c r="F10" s="6" t="str">
+        <x:v>Attempt Salary, Finance Worker money, and direct worker-money mutations.</x:v>
+      </x:c>
+      <x:c r="G10" s="6" t="str">
+        <x:v>Salary/worker-money data and commands remain denied; owner/admin and finance access continue.</x:v>
+      </x:c>
+      <x:c r="H10" s="6" t="str"/>
+      <x:c r="I10" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J10" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K10" s="6" t="str"/>
+    </x:row>
+    <x:row r="11" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A11" s="6" t="str">
+        <x:v>SA-010</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="str">
+        <x:v>Owner/Admin</x:v>
+      </x:c>
+      <x:c r="D11" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E11" s="6" t="str">
+        <x:v>Legacy deduction/repayment rows exist without an account or payment mode.</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="str">
+        <x:v>Open Salary Worker ledger, Finance Worker money, and Worker details.</x:v>
+      </x:c>
+      <x:c r="G11" s="6" t="str">
+        <x:v>Legacy rows remain visible as unallocated/Not recorded and are not silently reclassified or deleted.</x:v>
+      </x:c>
+      <x:c r="H11" s="6" t="str"/>
+      <x:c r="I11" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J11" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K11" s="6" t="str"/>
+    </x:row>
+    <x:row r="12" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>SA-011</x:v>
+      </x:c>
+      <x:c r="B12" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C12" s="6" t="str">
+        <x:v>Owner/Admin</x:v>
+      </x:c>
+      <x:c r="D12" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E12" s="6" t="str">
+        <x:v>More than 50 worker-ledger entries exist across multiple workers, including inactive worker history.</x:v>
+      </x:c>
+      <x:c r="F12" s="6" t="str">
+        <x:v>Open Worker ledger, filter one worker, then open that worker's details and page through history.</x:v>
+      </x:c>
+      <x:c r="G12" s="6" t="str">
+        <x:v>New entries appear immediately; inactive names remain resolved; database-calculated advance, loan, and salary-paid totals reconcile; every history row is reachable without tenant-wide truncation.</x:v>
+      </x:c>
+      <x:c r="H12" s="6" t="str"/>
+      <x:c r="I12" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J12" s="6" t="str">
+        <x:v>Database + Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K12" s="6" t="str"/>
+    </x:row>
+    <x:row r="13" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A13" s="6" t="str">
+        <x:v>SA-012</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="str">
+        <x:v>Owner/Admin or Finance</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E13" s="6" t="str">
+        <x:v>A worker-money form is open and valid tenant records exist.</x:v>
+      </x:c>
+      <x:c r="F13" s="6" t="str">
+        <x:v>Submit malformed dates/IDs, an over-balance amount, and two concurrent correction retries.</x:v>
+      </x:c>
+      <x:c r="G13" s="6" t="str">
+        <x:v>Each error is announced inline while input remains available; pending controls block duplicate interaction; no partial row is created; concurrent retries return one replacement and the next successful command uses a fresh idempotency key.</x:v>
+      </x:c>
+      <x:c r="H13" s="6" t="str"/>
+      <x:c r="I13" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J13" s="6" t="str">
+        <x:v>Database + Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K13" s="6" t="str"/>
+    </x:row>
+    <x:row r="14" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A14" s="6" t="str">
+        <x:v>SA-013</x:v>
+      </x:c>
+      <x:c r="B14" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C14" s="6" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="D14" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E14" s="6" t="str">
+        <x:v>Active workers exist and the disposable database has no period in the target range.</x:v>
+      </x:c>
+      <x:c r="F14" s="6" t="str">
+        <x:v>Preview a date range, change dates and verify confirmation invalidates, refresh preview, then create; retry after changing live generated inputs and force an invalid payload during regeneration.</x:v>
+      </x:c>
+      <x:c r="G14" s="6" t="str">
+        <x:v>Preview writes nothing and reports worker/attendance coverage plus suggested total. Confirmation requires the unchanged server fingerprint. A lost-response retry returns the original result without rewriting rows; invalid regeneration preserves the prior draft atomically.</x:v>
+      </x:c>
+      <x:c r="H14" s="6" t="str"/>
+      <x:c r="I14" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J14" s="6" t="str">
+        <x:v>Database + Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K14" s="6" t="str"/>
+    </x:row>
+    <x:row r="15" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A15" s="6" t="str">
+        <x:v>SA-014</x:v>
+      </x:c>
+      <x:c r="B15" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C15" s="6" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="D15" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E15" s="6" t="str">
+        <x:v>Two concurrent requests use different but overlapping ranges.</x:v>
+      </x:c>
+      <x:c r="F15" s="6" t="str">
+        <x:v>Submit both salary-period creates concurrently.</x:v>
+      </x:c>
+      <x:c r="G15" s="6" t="str">
+        <x:v>The tenant lock serializes both commands; exactly one period is created and the other returns the overlap error without partial calculations.</x:v>
+      </x:c>
+      <x:c r="H15" s="6" t="str"/>
+      <x:c r="I15" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J15" s="6" t="str">
+        <x:v>Database + Automated</x:v>
+      </x:c>
+      <x:c r="K15" s="6" t="str"/>
+    </x:row>
+    <x:row r="16" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A16" s="6" t="str">
+        <x:v>SA-015</x:v>
+      </x:c>
+      <x:c r="B16" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C16" s="6" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="D16" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E16" s="6" t="str">
+        <x:v>A draft period has no finalized or paid worker rows.</x:v>
+      </x:c>
+      <x:c r="F16" s="6" t="str">
+        <x:v>Edit the start/end dates, then finalize one worker and attempt another date edit.</x:v>
+      </x:c>
+      <x:c r="G16" s="6" t="str">
+        <x:v>Before decisions, dates and recalculated suggestions update atomically and the period remains selected. After any decision/payment, date editing and regeneration are unavailable and the database rejects stale attempts.</x:v>
+      </x:c>
+      <x:c r="H16" s="6" t="str"/>
+      <x:c r="I16" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J16" s="6" t="str">
+        <x:v>Database + Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K16" s="6" t="str"/>
+    </x:row>
+    <x:row r="17" ht="66" hidden="0" customHeight="1">
+      <x:c r="A17" s="6" t="str">
+        <x:v>SA-016</x:v>
+      </x:c>
+      <x:c r="B17" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C17" s="6" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="D17" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E17" s="6" t="str">
+        <x:v>One worker has a zero final payable; another has a partial payment.</x:v>
+      </x:c>
+      <x:c r="F17" s="6" t="str">
+        <x:v>Finalize zero payable, then attempt to lower the other worker's final payable below amount already paid.</x:v>
+      </x:c>
+      <x:c r="G17" s="6" t="str">
+        <x:v>Zero payable is shown as paid with No payment due. Final payable cannot be lower than paid; the rejected edit writes no audit revision and instructs the user to correct/reverse payment first.</x:v>
+      </x:c>
+      <x:c r="H17" s="6" t="str"/>
+      <x:c r="I17" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J17" s="6" t="str">
+        <x:v>Database + Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K17" s="6" t="str"/>
+    </x:row>
+    <x:row r="18" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A18" s="6" t="str">
+        <x:v>SA-017</x:v>
+      </x:c>
+      <x:c r="B18" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C18" s="6" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="D18" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E18" s="6" t="str">
+        <x:v>A period has two finalized workers with amounts due and an active payment mode exists.</x:v>
+      </x:c>
+      <x:c r="F18" s="6" t="str">
+        <x:v>Record concurrent final payments for different workers, then correct or reverse one payment and record the corrected balance.</x:v>
+      </x:c>
+      <x:c r="G18" s="6" t="str">
+        <x:v>Parent-period locking leaves the period Paid after concurrent settlement and Partially paid/Ready to pay after reopening as appropriate. Original and replacement evidence remains visible with actor/time/reason, and Finance refreshes each cash movement exactly once.</x:v>
+      </x:c>
+      <x:c r="H18" s="6" t="str"/>
+      <x:c r="I18" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J18" s="6" t="str">
+        <x:v>Database + Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K18" s="6" t="str"/>
+    </x:row>
+    <x:row r="19" ht="66" hidden="0" customHeight="1">
+      <x:c r="A19" s="6" t="str">
+        <x:v>SA-018</x:v>
+      </x:c>
+      <x:c r="B19" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C19" s="6" t="str">
+        <x:v>Owner/Admin or Finance</x:v>
+      </x:c>
+      <x:c r="D19" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E19" s="6" t="str">
+        <x:v>A worker payable has been finalized or updated more than once.</x:v>
+      </x:c>
+      <x:c r="F19" s="6" t="str">
+        <x:v>Open the worker row in its period and expand Payable decision history.</x:v>
+      </x:c>
+      <x:c r="G19" s="6" t="str">
+        <x:v>Immutable before/after payable values, reason, actor/time evidence, and payment history are visible. Server validation errors remain inline and do not navigate to a runtime error page.</x:v>
+      </x:c>
+      <x:c r="H19" s="6" t="str"/>
+      <x:c r="I19" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J19" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K19" s="6" t="str"/>
+    </x:row>
+    <x:row r="20" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A20" s="6" t="str">
+        <x:v>SA-019</x:v>
+      </x:c>
+      <x:c r="B20" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C20" s="6" t="str">
+        <x:v>Owner/Admin or Finance</x:v>
+      </x:c>
+      <x:c r="D20" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E20" s="6" t="str">
+        <x:v>A draft period contains two or more worker calculations, including one changed payable requiring a note.</x:v>
+      </x:c>
+      <x:c r="F20" s="6" t="str">
+        <x:v>Open the period workspace, select eligible workers, edit one payable/note, and finalize the selected rows; repeat the idempotency key and retry once with a stale or invalid selected row.</x:v>
+      </x:c>
+      <x:c r="G20" s="6" t="str">
+        <x:v>The full-width table shows every worker and filters; the valid batch commits once with one immutable revision per worker; retry returns the receipt; any stale/invalid row rejects the complete batch with preserved input and no partial decisions.</x:v>
+      </x:c>
+      <x:c r="H20" s="6" t="str"/>
+      <x:c r="I20" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J20" s="6" t="str">
+        <x:v>Database + Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K20" s="6" t="str"/>
+    </x:row>
+    <x:row r="21" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A21" s="6" t="str">
+        <x:v>SA-020</x:v>
+      </x:c>
+      <x:c r="B21" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C21" s="6" t="str">
+        <x:v>Owner/Admin or Finance</x:v>
+      </x:c>
+      <x:c r="D21" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E21" s="6" t="str">
+        <x:v>A period contains at least two finalized workers with outstanding salary and an active payment mode.</x:v>
+      </x:c>
+      <x:c r="F21" s="6" t="str">
+        <x:v>Select both workers in Record payments, use one date/mode, change one row to a partial amount, and submit; retry and repeat with one overpaying/stale row.</x:v>
+      </x:c>
+      <x:c r="G21" s="6" t="str">
+        <x:v>The valid batch creates one independently auditable salary-paid ledger row per worker and refreshes Salary, Finance, and Workers; retry does not duplicate cash; any invalid row rejects the complete batch. Mobile rows and sticky action remain usable at 320px.</x:v>
+      </x:c>
+      <x:c r="H21" s="6" t="str"/>
+      <x:c r="I21" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J21" s="6" t="str">
+        <x:v>Database + Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K21" s="6" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03e0ce6f94884bca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e7a69d768c745c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1797,10 +2328,70 @@
       </x:c>
       <x:c r="K4" s="6" t="str"/>
     </x:row>
+    <x:row r="5" ht="66" hidden="0" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>FI-004</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E5" s="6" t="str">
+        <x:v>Worker salary, advance, loan, repayment, deduction, and credit entries exist in the selected range.</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="str">
+        <x:v>Compare Finance Dashboard, Cashflow, and Worker money.</x:v>
+      </x:c>
+      <x:c r="G5" s="6" t="str">
+        <x:v>Salary/advance/loan count once as cash out; repayment counts once as cash in; deduction/credit are visible but excluded from cash totals; P&amp;L salary expense remains salary-only.</x:v>
+      </x:c>
+      <x:c r="H5" s="6" t="str"/>
+      <x:c r="I5" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J5" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K5" s="6" t="str"/>
+    </x:row>
+    <x:row r="6" ht="66" hidden="0" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>FI-005</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="str">
+        <x:v>Tenant A and Tenant B have workers, payment modes, and ledger entries.</x:v>
+      </x:c>
+      <x:c r="E6" s="6" t="str">
+        <x:v>Attempt record/correct/reverse using cross-tenant worker, mode, period, or entry IDs.</x:v>
+      </x:c>
+      <x:c r="F6" s="6" t="str">
+        <x:v>Every command fails without partial rows, balance changes, or Finance changes in either tenant.</x:v>
+      </x:c>
+      <x:c r="G6" s="6" t="str"/>
+      <x:c r="H6" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="I6" s="6" t="str">
+        <x:v>Database + Automated</x:v>
+      </x:c>
+      <x:c r="J6" s="6" t="str"/>
+      <x:c r="K6" s="6"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6710e9e338f243e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e0dc8164107469f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1984,7 +2575,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70318252ea184232"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4eafe91d34c433e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2137,7 +2728,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f72d013c5c742c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69c8f632f1e44290"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2292,7 +2883,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54a2d81de595426d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2be687680e14186"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2445,7 +3036,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a15f33e035543bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69534148a3274b59"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2629,7 +3220,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f5b06120f4d4a04"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1c1605cda1346a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2819,7 +3410,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62cf54a600bb411a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad8737f477d1429d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2985,15 +3576,15 @@
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E5" s="6" t="str">
-        <x:v>CSV and XLSX customer fixtures contain valid Indian, explicit international, country-assisted foreign, ambiguous foreign, blank-name, malformed, and over-limit cases.</x:v>
+        <x:v>CSV and XLSX customer fixtures contain valid Indian, explicit international, country-assisted foreign, unverified foreign, blank-name, malformed, and over-limit cases.</x:v>
       </x:c>
       <x:c r="F5" s="6" t="str">
         <x:v>Preview each file, including files larger than 5 MB or 5,000 data rows.</x:v>
       </x:c>
       <x:c r="G5" s="6" t="str">
-        <x:v>Valid rows preview without writes; foreign numbers normalize only with explicit/country context; ambiguous phones, blank names, malformed files, and limits are rejected or counted; the invalid/skipped count is visible.</x:v>
-      </x:c>
-      <x:c r="H5" s="6" t="str"/>
+        <x:v>Valid rows preview without writes; foreign numbers normalize only with explicit/country context; plausible unverified phones require review or an authoritative Shopify ID and never become match keys; blank names, malformed files, and limits are rejected or counted; review and invalid/skipped counts are visible.</x:v>
+      </x:c>
+      <x:c r="H5" s="6"/>
       <x:c r="I5" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
@@ -3103,10 +3694,43 @@
         <x:v>Metadata is a future Shopify-integration foundation only.</x:v>
       </x:c>
     </x:row>
+    <x:row r="9" ht="135" hidden="0" customHeight="1">
+      <x:c r="A9" s="1" t="str">
+        <x:v>CU-008</x:v>
+      </x:c>
+      <x:c r="B9" s="1" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C9" s="1" t="str">
+        <x:v>Owner/Admin</x:v>
+      </x:c>
+      <x:c r="D9" s="1" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E9" s="1" t="str">
+        <x:v>Rows contain valid US/Australian/Indian numbers, differing Shopify Phone/address-phone values, plausible unverified 7-to-15-digit values, and too-short values.</x:v>
+      </x:c>
+      <x:c r="F9" s="1" t="str">
+        <x:v>Preview the file, resolve an unverified row without Shopify ID, and confirm approved rows.</x:v>
+      </x:c>
+      <x:c r="G9" s="1" t="str">
+        <x:v>Valid country-resolved numbers normalize to E.164; Shopify Phone remains primary; a differing address phone is warning-only metadata; unverified values never match by phone; no-ID unverified rows require Create without verified phone or Skip; too-short values remain invalid.</x:v>
+      </x:c>
+      <x:c r="H9" s="1"/>
+      <x:c r="I9" s="1" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J9" s="1" t="str">
+        <x:v>Automated + Manual</x:v>
+      </x:c>
+      <x:c r="K9" s="1" t="str">
+        <x:v>No database migration is required; alternate and unverified values remain Shopify identity metadata only.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43412d8656404228"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e5a382a2aa54eea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3259,7 +3883,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R969d71460bb4493a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ea70c2699f1423b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3659,10 +4283,43 @@
       </x:c>
       <x:c r="K12" s="6" t="str"/>
     </x:row>
+    <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A13" s="6" t="str">
+        <x:v>CF-012</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="str">
+        <x:v>Owner/Admin</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E13" s="6" t="str">
+        <x:v>An item type uses an assignment-only stage.</x:v>
+      </x:c>
+      <x:c r="F13" s="6" t="str">
+        <x:v>Open that item type's Contribution rules.</x:v>
+      </x:c>
+      <x:c r="G13" s="6" t="str">
+        <x:v>The row explains that effort tracking is required and links to stage configuration instead of silently hiding the action.</x:v>
+      </x:c>
+      <x:c r="H13" s="6" t="str"/>
+      <x:c r="I13" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J13" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K13" s="6" t="str">
+        <x:v>No incompatible monetary rule is offered.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea9e623bcefc4389"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra62151d40b6e4818"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3881,7 +4538,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cb1abe9b6f342d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98723884fe84425d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4482,7 +5139,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d8755ad1983420b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R010d27a191974be9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4637,7 +5294,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6c6c7466c6a4b51"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1bebfab68a544b88"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>